<commit_message>
added the Secure Settings - Categorize Options procedure material
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCDL tool cybersecurity options template.xlsx
+++ b/distribution/reference_documents/templates/AVCDL tool cybersecurity options template.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B145337-C499-6846-8774-5329695E90AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C71A2E1-95C7-CF40-AF23-0B40FA017BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30840" yWindow="6440" windowWidth="26580" windowHeight="22600" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
+    <workbookView xWindow="35680" yWindow="9460" windowWidth="35800" windowHeight="22600" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="7" r:id="rId1"/>
     <sheet name="revision history" sheetId="9" r:id="rId2"/>
     <sheet name="references" sheetId="10" r:id="rId3"/>
     <sheet name="options" sheetId="6" r:id="rId4"/>
-    <sheet name="legend" sheetId="2" r:id="rId5"/>
+    <sheet name="categories" sheetId="16" r:id="rId5"/>
+    <sheet name="legend" sheetId="2" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>DO NOT EDIT THIS PAGE</t>
   </si>
@@ -164,6 +165,15 @@
   </si>
   <si>
     <t>Tool Platform</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>qualifications</t>
+  </si>
+  <si>
+    <t>category</t>
   </si>
 </sst>
 </file>
@@ -1108,17 +1118,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F77D532C-C0F7-A74D-BEFF-3C27CE960CDF}">
-  <dimension ref="A2:J20"/>
+  <dimension ref="A2:K20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.5" customWidth="1"/>
     <col min="4" max="4" width="26.5" customWidth="1"/>
     <col min="5" max="5" width="27.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="7" max="8" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" ht="63" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:11" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="27" t="s">
         <v>33</v>
       </c>
@@ -1127,11 +1137,12 @@
       <c r="E2" s="27"/>
       <c r="F2" s="27"/>
       <c r="G2" s="27"/>
-      <c r="H2" s="7"/>
+      <c r="H2" s="27"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" s="7"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
         <v>1</v>
@@ -1149,151 +1160,176 @@
         <v>32</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="5"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="5"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="5"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="5"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="5"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="5"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="5"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="5"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="5"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="5"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="5"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="5"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="5"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="5"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="5"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="1">
-    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BACB055F-480B-4F40-91CA-D13E071195DD}">
           <x14:formula1>
             <xm:f>legend!$A$2:$A$10</xm:f>
           </x14:formula1>
           <xm:sqref>F5:F20</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0C95FE9F-B4FC-5E49-BDF1-B78B4A9307E2}">
+          <x14:formula1>
+            <xm:f>categories!$C$13:$C$20</xm:f>
+          </x14:formula1>
+          <xm:sqref>G5:G20</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1302,6 +1338,168 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB364F2E-B8A7-6640-86AB-62A730DA1093}">
+  <dimension ref="A2:I20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="11.5" customWidth="1"/>
+    <col min="4" max="4" width="26.5" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" ht="63" x14ac:dyDescent="0.75">
+      <c r="B2" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+  </sheetData>
+  <dataConsolidate/>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34E47EDA-BFD6-E448-BD76-322D521CE805}">
   <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1409,7 +1607,7 @@
         <v>5</v>
       </c>
       <c r="D29" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G29" s="10"/>
       <c r="H29" s="11"/>

</xml_diff>